<commit_message>
v2: social, presentation, documents, cards and signatures rebuilt on the new system with real contacts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLSMnj5wd3Rg3Zvu6XTEmR
</commit_message>
<xml_diff>
--- a/DESTINATION-NIGERIA-BRAND-KIT/09_DOCUMENT_TEMPLATES/INVOICES/DN_Invoice_Template_A4.xlsx
+++ b/DESTINATION-NIGERIA-BRAND-KIT/09_DOCUMENT_TEMPLATES/INVOICES/DN_Invoice_Template_A4.xlsx
@@ -28,43 +28,43 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Playfair Display"/>
+      <name val="Newsreader Display"/>
       <color rgb="00103428"/>
       <sz val="22"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <b val="1"/>
       <color rgb="00103428"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <color rgb="005F6662"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <color rgb="00103428"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <b val="1"/>
       <color rgb="00103428"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Inter"/>
+      <name val="Public Sans"/>
       <color rgb="005F6662"/>
       <sz val="8"/>
     </font>

</xml_diff>